<commit_message>
added multiple stop time
</commit_message>
<xml_diff>
--- a/style/sample_excels/bulk_bus_master_upload.xlsx
+++ b/style/sample_excels/bulk_bus_master_upload.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buses" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busses" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -38,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,13 +46,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,8 +437,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -434,67 +461,190 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Stop Order</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Stop Name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Timing</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Capacity</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Stops</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>RC Bus 1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Dadar (Swaminarayan Temple)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="D2" t="n">
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RC Bus 1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Dadar | Airoli | Research Centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Airoli</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>RC Bus 1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Borivali (Indraprasth Shopping Centre)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>RC Bus 1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Research Centre</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Airport Bus</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Research Centre | Airport Terminal 2</t>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Airport Terminal 2</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Airport Bus</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Research Centre</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
         </is>
       </c>
     </row>
@@ -511,6 +661,10 @@
   </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -525,36 +679,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>RC Bus 1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>BK001</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>RC Bus 1</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>BK002</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Airport Bus</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>BK003</t>
         </is>

</xml_diff>